<commit_message>
benchmark all models by hyperparameters, lookbacks, kernel-filter for CNN-LSTM model
</commit_message>
<xml_diff>
--- a/src_code/outputs/SC3_results.xlsx
+++ b/src_code/outputs/SC3_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,7 +486,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -500,28 +500,28 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F2" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G2" t="n">
-        <v>0.268</v>
+        <v>0.3548</v>
       </c>
       <c r="H2" t="n">
-        <v>0.183</v>
+        <v>0.2383</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7045</v>
+        <v>0.4823</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2217</v>
+        <v>0.2938</v>
       </c>
       <c r="K2" t="n">
-        <v>0.1709</v>
+        <v>0.2273</v>
       </c>
       <c r="L2" t="n">
-        <v>0.9105</v>
+        <v>0.8428</v>
       </c>
     </row>
     <row r="3">
@@ -532,7 +532,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -546,28 +546,28 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3378</v>
+        <v>0.3183</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2197</v>
+        <v>0.21</v>
       </c>
       <c r="I3" t="n">
-        <v>0.5298</v>
+        <v>0.5818</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2577</v>
+        <v>0.2813</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1957</v>
+        <v>0.2151</v>
       </c>
       <c r="L3" t="n">
-        <v>0.879</v>
+        <v>0.8556</v>
       </c>
     </row>
     <row r="4">
@@ -578,7 +578,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -592,28 +592,28 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F4" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3266</v>
+        <v>0.3348</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2123</v>
+        <v>0.2129</v>
       </c>
       <c r="I4" t="n">
-        <v>0.5601</v>
+        <v>0.5343</v>
       </c>
       <c r="J4" t="n">
-        <v>0.265</v>
+        <v>0.3305</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1996</v>
+        <v>0.2511</v>
       </c>
       <c r="L4" t="n">
-        <v>0.872</v>
+        <v>0.7995</v>
       </c>
     </row>
     <row r="5">
@@ -624,7 +624,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -638,28 +638,28 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2143</v>
+        <v>0.3006</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1475</v>
+        <v>0.1891</v>
       </c>
       <c r="I5" t="n">
-        <v>0.8101</v>
+        <v>0.6272</v>
       </c>
       <c r="J5" t="n">
-        <v>0.1974</v>
+        <v>0.2691</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1521</v>
+        <v>0.202</v>
       </c>
       <c r="L5" t="n">
-        <v>0.9288999999999999</v>
+        <v>0.868</v>
       </c>
     </row>
     <row r="6">
@@ -670,7 +670,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -684,28 +684,28 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2228</v>
+        <v>0.2702</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1513</v>
+        <v>0.1726</v>
       </c>
       <c r="I6" t="n">
-        <v>0.7944</v>
+        <v>0.6979</v>
       </c>
       <c r="J6" t="n">
-        <v>0.2084</v>
+        <v>0.2755</v>
       </c>
       <c r="K6" t="n">
-        <v>0.1581</v>
+        <v>0.2079</v>
       </c>
       <c r="L6" t="n">
-        <v>0.9207</v>
+        <v>0.8612</v>
       </c>
     </row>
     <row r="7">
@@ -716,7 +716,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -730,28 +730,28 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2319</v>
+        <v>0.3161</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1603</v>
+        <v>0.2014</v>
       </c>
       <c r="I7" t="n">
-        <v>0.777</v>
+        <v>0.5835</v>
       </c>
       <c r="J7" t="n">
-        <v>0.2173</v>
+        <v>0.3157</v>
       </c>
       <c r="K7" t="n">
-        <v>0.1648</v>
+        <v>0.2397</v>
       </c>
       <c r="L7" t="n">
-        <v>0.9137</v>
+        <v>0.8168</v>
       </c>
     </row>
     <row r="8">
@@ -762,7 +762,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -776,28 +776,28 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="F8" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2048</v>
+        <v>0.2393</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1412</v>
+        <v>0.1576</v>
       </c>
       <c r="I8" t="n">
-        <v>0.8247</v>
+        <v>0.7627</v>
       </c>
       <c r="J8" t="n">
-        <v>0.1902</v>
+        <v>0.2445</v>
       </c>
       <c r="K8" t="n">
-        <v>0.146</v>
+        <v>0.1853</v>
       </c>
       <c r="L8" t="n">
-        <v>0.9336</v>
+        <v>0.8907</v>
       </c>
     </row>
     <row r="9">
@@ -808,7 +808,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -822,28 +822,28 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="F9" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2243</v>
+        <v>0.2335</v>
       </c>
       <c r="H9" t="n">
-        <v>0.15</v>
+        <v>0.1548</v>
       </c>
       <c r="I9" t="n">
-        <v>0.7896</v>
+        <v>0.7731</v>
       </c>
       <c r="J9" t="n">
-        <v>0.2046</v>
+        <v>0.2527</v>
       </c>
       <c r="K9" t="n">
-        <v>0.1539</v>
+        <v>0.1889</v>
       </c>
       <c r="L9" t="n">
-        <v>0.9231</v>
+        <v>0.8829</v>
       </c>
     </row>
     <row r="10">
@@ -854,7 +854,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -868,28 +868,28 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="F10" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2306</v>
+        <v>0.2938</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1594</v>
+        <v>0.1936</v>
       </c>
       <c r="I10" t="n">
-        <v>0.7774</v>
+        <v>0.6383</v>
       </c>
       <c r="J10" t="n">
-        <v>0.2116</v>
+        <v>0.3666</v>
       </c>
       <c r="K10" t="n">
-        <v>0.1612</v>
+        <v>0.2631</v>
       </c>
       <c r="L10" t="n">
-        <v>0.9177</v>
+        <v>0.7523</v>
       </c>
     </row>
     <row r="11">
@@ -900,7 +900,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -910,32 +910,32 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>LSTM</t>
+          <t>RNN</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="F11" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2511</v>
+        <v>0.2323</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1588</v>
+        <v>0.1582</v>
       </c>
       <c r="I11" t="n">
-        <v>0.7405</v>
+        <v>0.7739</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2118</v>
+        <v>0.2339</v>
       </c>
       <c r="K11" t="n">
-        <v>0.1568</v>
+        <v>0.1753</v>
       </c>
       <c r="L11" t="n">
-        <v>0.9184</v>
+        <v>0.8995</v>
       </c>
     </row>
     <row r="12">
@@ -946,7 +946,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -956,32 +956,32 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>LSTM</t>
+          <t>RNN</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="F12" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G12" t="n">
-        <v>0.3116</v>
+        <v>0.2499</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1948</v>
+        <v>0.1736</v>
       </c>
       <c r="I12" t="n">
-        <v>0.5999</v>
+        <v>0.7375</v>
       </c>
       <c r="J12" t="n">
-        <v>0.2456</v>
+        <v>0.2523</v>
       </c>
       <c r="K12" t="n">
-        <v>0.1814</v>
+        <v>0.194</v>
       </c>
       <c r="L12" t="n">
-        <v>0.8901</v>
+        <v>0.8827</v>
       </c>
     </row>
     <row r="13">
@@ -992,7 +992,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1002,32 +1002,32 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>LSTM</t>
+          <t>RNN</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="F13" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="G13" t="n">
-        <v>0.33</v>
+        <v>0.3014</v>
       </c>
       <c r="H13" t="n">
-        <v>0.2052</v>
+        <v>0.2028</v>
       </c>
       <c r="I13" t="n">
-        <v>0.5508999999999999</v>
+        <v>0.6153999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>0.2594</v>
+        <v>0.3208</v>
       </c>
       <c r="K13" t="n">
-        <v>0.1932</v>
+        <v>0.2416</v>
       </c>
       <c r="L13" t="n">
-        <v>0.8773</v>
+        <v>0.8093</v>
       </c>
     </row>
     <row r="14">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1052,28 +1052,28 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="F14" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1876</v>
+        <v>0.3314</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1209</v>
+        <v>0.2248</v>
       </c>
       <c r="I14" t="n">
-        <v>0.8545</v>
+        <v>0.5481</v>
       </c>
       <c r="J14" t="n">
-        <v>0.1765</v>
+        <v>0.3204</v>
       </c>
       <c r="K14" t="n">
-        <v>0.1292</v>
+        <v>0.2511</v>
       </c>
       <c r="L14" t="n">
-        <v>0.9431</v>
+        <v>0.8129999999999999</v>
       </c>
     </row>
     <row r="15">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1098,28 +1098,28 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="F15" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2106</v>
+        <v>0.3057</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1331</v>
+        <v>0.2022</v>
       </c>
       <c r="I15" t="n">
-        <v>0.8163</v>
+        <v>0.6142</v>
       </c>
       <c r="J15" t="n">
-        <v>0.2007</v>
+        <v>0.3134</v>
       </c>
       <c r="K15" t="n">
-        <v>0.1481</v>
+        <v>0.2411</v>
       </c>
       <c r="L15" t="n">
-        <v>0.9264</v>
+        <v>0.8207</v>
       </c>
     </row>
     <row r="16">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1144,28 +1144,28 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="F16" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="G16" t="n">
-        <v>0.2832</v>
+        <v>0.3319</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1862</v>
+        <v>0.2136</v>
       </c>
       <c r="I16" t="n">
-        <v>0.6676</v>
+        <v>0.5421</v>
       </c>
       <c r="J16" t="n">
-        <v>0.2946</v>
+        <v>0.3691</v>
       </c>
       <c r="K16" t="n">
-        <v>0.2285</v>
+        <v>0.2787</v>
       </c>
       <c r="L16" t="n">
-        <v>0.8413</v>
+        <v>0.7499</v>
       </c>
     </row>
     <row r="17">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1190,28 +1190,28 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="F17" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1908</v>
+        <v>0.3196</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1235</v>
+        <v>0.21</v>
       </c>
       <c r="I17" t="n">
-        <v>0.8479</v>
+        <v>0.5788</v>
       </c>
       <c r="J17" t="n">
-        <v>0.1802</v>
+        <v>0.2895</v>
       </c>
       <c r="K17" t="n">
-        <v>0.1323</v>
+        <v>0.2197</v>
       </c>
       <c r="L17" t="n">
-        <v>0.9404</v>
+        <v>0.8472</v>
       </c>
     </row>
     <row r="18">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1236,28 +1236,28 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="F18" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G18" t="n">
-        <v>0.2091</v>
+        <v>0.2732</v>
       </c>
       <c r="H18" t="n">
-        <v>0.137</v>
+        <v>0.171</v>
       </c>
       <c r="I18" t="n">
-        <v>0.8172</v>
+        <v>0.6909999999999999</v>
       </c>
       <c r="J18" t="n">
-        <v>0.2039</v>
+        <v>0.2831</v>
       </c>
       <c r="K18" t="n">
-        <v>0.1497</v>
+        <v>0.2082</v>
       </c>
       <c r="L18" t="n">
-        <v>0.9237</v>
+        <v>0.8535</v>
       </c>
     </row>
     <row r="19">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1282,28 +1282,28 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="F19" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="G19" t="n">
-        <v>0.2169</v>
+        <v>0.3143</v>
       </c>
       <c r="H19" t="n">
-        <v>0.1358</v>
+        <v>0.2001</v>
       </c>
       <c r="I19" t="n">
-        <v>0.8028999999999999</v>
+        <v>0.5884</v>
       </c>
       <c r="J19" t="n">
-        <v>0.2194</v>
+        <v>0.4161</v>
       </c>
       <c r="K19" t="n">
-        <v>0.1572</v>
+        <v>0.2836</v>
       </c>
       <c r="L19" t="n">
-        <v>0.9116</v>
+        <v>0.6819</v>
       </c>
     </row>
     <row r="20">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1324,32 +1324,32 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>GRU</t>
+          <t>LSTM</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F20" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G20" t="n">
-        <v>0.2499</v>
+        <v>0.2374</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1605</v>
+        <v>0.1622</v>
       </c>
       <c r="I20" t="n">
-        <v>0.7431</v>
+        <v>0.7664</v>
       </c>
       <c r="J20" t="n">
-        <v>0.2145</v>
+        <v>0.2547</v>
       </c>
       <c r="K20" t="n">
-        <v>0.1597</v>
+        <v>0.1918</v>
       </c>
       <c r="L20" t="n">
-        <v>0.9162</v>
+        <v>0.8814</v>
       </c>
     </row>
     <row r="21">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1370,32 +1370,32 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>GRU</t>
+          <t>LSTM</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F21" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G21" t="n">
-        <v>0.3055</v>
+        <v>0.2387</v>
       </c>
       <c r="H21" t="n">
-        <v>0.1891</v>
+        <v>0.1595</v>
       </c>
       <c r="I21" t="n">
-        <v>0.6156</v>
+        <v>0.763</v>
       </c>
       <c r="J21" t="n">
-        <v>0.248</v>
+        <v>0.2867</v>
       </c>
       <c r="K21" t="n">
-        <v>0.1849</v>
+        <v>0.2101</v>
       </c>
       <c r="L21" t="n">
-        <v>0.888</v>
+        <v>0.8493000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1416,32 +1416,32 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>GRU</t>
+          <t>LSTM</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F22" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="G22" t="n">
-        <v>0.328</v>
+        <v>0.2864</v>
       </c>
       <c r="H22" t="n">
-        <v>0.2082</v>
+        <v>0.1856</v>
       </c>
       <c r="I22" t="n">
-        <v>0.5562</v>
+        <v>0.6565</v>
       </c>
       <c r="J22" t="n">
-        <v>0.263</v>
+        <v>0.4265</v>
       </c>
       <c r="K22" t="n">
-        <v>0.1967</v>
+        <v>0.2893</v>
       </c>
       <c r="L22" t="n">
-        <v>0.8739</v>
+        <v>0.6649</v>
       </c>
     </row>
     <row r="23">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1462,32 +1462,32 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>GRU</t>
+          <t>LSTM</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="F23" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G23" t="n">
-        <v>0.1937</v>
+        <v>0.226</v>
       </c>
       <c r="H23" t="n">
-        <v>0.1253</v>
+        <v>0.1539</v>
       </c>
       <c r="I23" t="n">
-        <v>0.8448</v>
+        <v>0.7861</v>
       </c>
       <c r="J23" t="n">
-        <v>0.1804</v>
+        <v>0.2517</v>
       </c>
       <c r="K23" t="n">
-        <v>0.1344</v>
+        <v>0.1947</v>
       </c>
       <c r="L23" t="n">
-        <v>0.9406</v>
+        <v>0.8836000000000001</v>
       </c>
     </row>
     <row r="24">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1508,32 +1508,32 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>GRU</t>
+          <t>LSTM</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="F24" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G24" t="n">
-        <v>0.235</v>
+        <v>0.2342</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1527</v>
+        <v>0.1628</v>
       </c>
       <c r="I24" t="n">
-        <v>0.7714</v>
+        <v>0.7694</v>
       </c>
       <c r="J24" t="n">
-        <v>0.2085</v>
+        <v>0.268</v>
       </c>
       <c r="K24" t="n">
-        <v>0.1565</v>
+        <v>0.1987</v>
       </c>
       <c r="L24" t="n">
-        <v>0.9206</v>
+        <v>0.8676</v>
       </c>
     </row>
     <row r="25">
@@ -1544,7 +1544,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1554,32 +1554,32 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GRU</t>
+          <t>LSTM</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="F25" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="G25" t="n">
-        <v>0.2336</v>
+        <v>0.2935</v>
       </c>
       <c r="H25" t="n">
-        <v>0.1493</v>
+        <v>0.1973</v>
       </c>
       <c r="I25" t="n">
-        <v>0.7738</v>
+        <v>0.6354</v>
       </c>
       <c r="J25" t="n">
-        <v>0.2138</v>
+        <v>0.4052</v>
       </c>
       <c r="K25" t="n">
-        <v>0.1593</v>
+        <v>0.2709</v>
       </c>
       <c r="L25" t="n">
-        <v>0.9165</v>
+        <v>0.6957</v>
       </c>
     </row>
     <row r="26">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1604,28 +1604,28 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="F26" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G26" t="n">
-        <v>0.1935</v>
+        <v>0.3318</v>
       </c>
       <c r="H26" t="n">
-        <v>0.1273</v>
+        <v>0.2186</v>
       </c>
       <c r="I26" t="n">
-        <v>0.8436</v>
+        <v>0.547</v>
       </c>
       <c r="J26" t="n">
-        <v>0.1812</v>
+        <v>0.314</v>
       </c>
       <c r="K26" t="n">
-        <v>0.134</v>
+        <v>0.2426</v>
       </c>
       <c r="L26" t="n">
-        <v>0.9397</v>
+        <v>0.8204</v>
       </c>
     </row>
     <row r="27">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1650,28 +1650,28 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="F27" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2254</v>
+        <v>0.3125</v>
       </c>
       <c r="H27" t="n">
-        <v>0.1468</v>
+        <v>0.1982</v>
       </c>
       <c r="I27" t="n">
-        <v>0.7875</v>
+        <v>0.597</v>
       </c>
       <c r="J27" t="n">
-        <v>0.2091</v>
+        <v>0.3088</v>
       </c>
       <c r="K27" t="n">
-        <v>0.1549</v>
+        <v>0.2361</v>
       </c>
       <c r="L27" t="n">
-        <v>0.9197</v>
+        <v>0.8259</v>
       </c>
     </row>
     <row r="28">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1696,28 +1696,28 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="F28" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="G28" t="n">
-        <v>0.2297</v>
+        <v>0.3605</v>
       </c>
       <c r="H28" t="n">
-        <v>0.154</v>
+        <v>0.2465</v>
       </c>
       <c r="I28" t="n">
-        <v>0.779</v>
+        <v>0.4598</v>
       </c>
       <c r="J28" t="n">
-        <v>0.2188</v>
+        <v>0.4025</v>
       </c>
       <c r="K28" t="n">
-        <v>0.1635</v>
+        <v>0.307</v>
       </c>
       <c r="L28" t="n">
-        <v>0.912</v>
+        <v>0.7026</v>
       </c>
     </row>
     <row r="29">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1738,32 +1738,32 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>CNN_LSTM</t>
+          <t>GRU</t>
         </is>
       </c>
       <c r="E29" t="n">
         <v>12</v>
       </c>
       <c r="F29" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G29" t="n">
-        <v>0.2666</v>
+        <v>0.3107</v>
       </c>
       <c r="H29" t="n">
-        <v>0.1707</v>
+        <v>0.1964</v>
       </c>
       <c r="I29" t="n">
-        <v>0.7074</v>
+        <v>0.6017</v>
       </c>
       <c r="J29" t="n">
-        <v>0.2321</v>
+        <v>0.2808</v>
       </c>
       <c r="K29" t="n">
-        <v>0.1771</v>
+        <v>0.2104</v>
       </c>
       <c r="L29" t="n">
-        <v>0.9019</v>
+        <v>0.8562</v>
       </c>
     </row>
     <row r="30">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1784,32 +1784,32 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CNN_LSTM</t>
+          <t>GRU</t>
         </is>
       </c>
       <c r="E30" t="n">
         <v>12</v>
       </c>
       <c r="F30" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G30" t="n">
-        <v>0.3013</v>
+        <v>0.2711</v>
       </c>
       <c r="H30" t="n">
-        <v>0.1888</v>
+        <v>0.1735</v>
       </c>
       <c r="I30" t="n">
-        <v>0.626</v>
+        <v>0.6959</v>
       </c>
       <c r="J30" t="n">
-        <v>0.2484</v>
+        <v>0.2845</v>
       </c>
       <c r="K30" t="n">
-        <v>0.1824</v>
+        <v>0.219</v>
       </c>
       <c r="L30" t="n">
-        <v>0.8875999999999999</v>
+        <v>0.852</v>
       </c>
     </row>
     <row r="31">
@@ -1820,7 +1820,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1830,32 +1830,32 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CNN_LSTM</t>
+          <t>GRU</t>
         </is>
       </c>
       <c r="E31" t="n">
         <v>12</v>
       </c>
       <c r="F31" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="G31" t="n">
-        <v>0.3079</v>
+        <v>0.3109</v>
       </c>
       <c r="H31" t="n">
-        <v>0.1942</v>
+        <v>0.1985</v>
       </c>
       <c r="I31" t="n">
-        <v>0.6089</v>
+        <v>0.5974</v>
       </c>
       <c r="J31" t="n">
-        <v>0.2487</v>
+        <v>0.3573</v>
       </c>
       <c r="K31" t="n">
-        <v>0.1852</v>
+        <v>0.2633</v>
       </c>
       <c r="L31" t="n">
-        <v>0.8872</v>
+        <v>0.7654</v>
       </c>
     </row>
     <row r="32">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1876,32 +1876,32 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>CNN_LSTM</t>
+          <t>GRU</t>
         </is>
       </c>
       <c r="E32" t="n">
         <v>24</v>
       </c>
       <c r="F32" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G32" t="n">
-        <v>0.1907</v>
+        <v>0.2339</v>
       </c>
       <c r="H32" t="n">
-        <v>0.1248</v>
+        <v>0.1579</v>
       </c>
       <c r="I32" t="n">
-        <v>0.8496</v>
+        <v>0.7731</v>
       </c>
       <c r="J32" t="n">
-        <v>0.1809</v>
+        <v>0.2488</v>
       </c>
       <c r="K32" t="n">
-        <v>0.1339</v>
+        <v>0.1882</v>
       </c>
       <c r="L32" t="n">
-        <v>0.9403</v>
+        <v>0.8868</v>
       </c>
     </row>
     <row r="33">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1922,32 +1922,32 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>CNN_LSTM</t>
+          <t>GRU</t>
         </is>
       </c>
       <c r="E33" t="n">
         <v>24</v>
       </c>
       <c r="F33" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G33" t="n">
-        <v>0.2142</v>
+        <v>0.2376</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1387</v>
+        <v>0.1539</v>
       </c>
       <c r="I33" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.7652</v>
       </c>
       <c r="J33" t="n">
-        <v>0.2111</v>
+        <v>0.2728</v>
       </c>
       <c r="K33" t="n">
-        <v>0.1535</v>
+        <v>0.1993</v>
       </c>
       <c r="L33" t="n">
-        <v>0.9186</v>
+        <v>0.8635</v>
       </c>
     </row>
     <row r="34">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1968,32 +1968,32 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>CNN_LSTM</t>
+          <t>GRU</t>
         </is>
       </c>
       <c r="E34" t="n">
         <v>24</v>
       </c>
       <c r="F34" t="n">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="G34" t="n">
-        <v>0.2262</v>
+        <v>0.2976</v>
       </c>
       <c r="H34" t="n">
-        <v>0.1465</v>
+        <v>0.1934</v>
       </c>
       <c r="I34" t="n">
-        <v>0.7879</v>
+        <v>0.629</v>
       </c>
       <c r="J34" t="n">
-        <v>0.2177</v>
+        <v>0.3551</v>
       </c>
       <c r="K34" t="n">
-        <v>0.1603</v>
+        <v>0.2626</v>
       </c>
       <c r="L34" t="n">
-        <v>0.9133</v>
+        <v>0.7677</v>
       </c>
     </row>
     <row r="35">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2014,32 +2014,32 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>CNN_LSTM</t>
+          <t>GRU</t>
         </is>
       </c>
       <c r="E35" t="n">
         <v>48</v>
       </c>
       <c r="F35" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G35" t="n">
-        <v>0.1884</v>
+        <v>0.2484</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1271</v>
+        <v>0.1661</v>
       </c>
       <c r="I35" t="n">
-        <v>0.8517</v>
+        <v>0.7417</v>
       </c>
       <c r="J35" t="n">
-        <v>0.1816</v>
+        <v>0.2531</v>
       </c>
       <c r="K35" t="n">
-        <v>0.136</v>
+        <v>0.1901</v>
       </c>
       <c r="L35" t="n">
-        <v>0.9395</v>
+        <v>0.8822</v>
       </c>
     </row>
     <row r="36">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2060,32 +2060,32 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>CNN_LSTM</t>
+          <t>GRU</t>
         </is>
       </c>
       <c r="E36" t="n">
         <v>48</v>
       </c>
       <c r="F36" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G36" t="n">
-        <v>0.2157</v>
+        <v>0.2365</v>
       </c>
       <c r="H36" t="n">
-        <v>0.1426</v>
+        <v>0.1592</v>
       </c>
       <c r="I36" t="n">
-        <v>0.8053</v>
+        <v>0.7649</v>
       </c>
       <c r="J36" t="n">
-        <v>0.2046</v>
+        <v>0.2711</v>
       </c>
       <c r="K36" t="n">
-        <v>0.1523</v>
+        <v>0.2004</v>
       </c>
       <c r="L36" t="n">
-        <v>0.9231</v>
+        <v>0.8646</v>
       </c>
     </row>
     <row r="37">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>BenLuc</t>
+          <t>BenLuc+CauNoi+TanAn</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2106,32 +2106,584 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
+          <t>GRU</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>48</v>
+      </c>
+      <c r="F37" t="n">
+        <v>48</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.3104</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.2009</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.5921999999999999</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.3509</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0.2567</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0.7719</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SC2</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>BenLuc+CauNoi+TanAn</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>BenLuc</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
           <t>CNN_LSTM</t>
         </is>
       </c>
-      <c r="E37" t="n">
-        <v>48</v>
-      </c>
-      <c r="F37" t="n">
-        <v>12</v>
-      </c>
-      <c r="G37" t="n">
-        <v>0.2396</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0.1586</v>
-      </c>
-      <c r="I37" t="n">
-        <v>0.7595</v>
-      </c>
-      <c r="J37" t="n">
-        <v>0.2111</v>
-      </c>
-      <c r="K37" t="n">
-        <v>0.1565</v>
-      </c>
-      <c r="L37" t="n">
-        <v>0.9181</v>
+      <c r="E38" t="n">
+        <v>6</v>
+      </c>
+      <c r="F38" t="n">
+        <v>12</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.3346</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.2188</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.5396</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.3314</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0.2536</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SC2</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>BenLuc+CauNoi+TanAn</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>BenLuc</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>6</v>
+      </c>
+      <c r="F39" t="n">
+        <v>24</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.3094</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.2015</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.605</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.3159</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0.2436</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0.8178</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SC2</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>BenLuc+CauNoi+TanAn</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>BenLuc</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>6</v>
+      </c>
+      <c r="F40" t="n">
+        <v>48</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.3435</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.2198</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.5096000000000001</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0.4021</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0.2966</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0.7032</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SC2</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>BenLuc+CauNoi+TanAn</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>BenLuc</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>12</v>
+      </c>
+      <c r="F41" t="n">
+        <v>12</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.3209</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.5753</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0.2955</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0.2206</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0.8408</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SC2</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>BenLuc+CauNoi+TanAn</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>BenLuc</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>12</v>
+      </c>
+      <c r="F42" t="n">
+        <v>24</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.2835</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.1833</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0.6674</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0.2988</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0.2204</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0.8368</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SC2</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>BenLuc+CauNoi+TanAn</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>BenLuc</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>12</v>
+      </c>
+      <c r="F43" t="n">
+        <v>48</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.319</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.2064</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.576</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.3861</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0.2766</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0.726</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SC2</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>BenLuc+CauNoi+TanAn</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>BenLuc</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>24</v>
+      </c>
+      <c r="F44" t="n">
+        <v>12</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.1732</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.7218</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0.2667</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0.2003</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SC2</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>BenLuc+CauNoi+TanAn</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>BenLuc</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>24</v>
+      </c>
+      <c r="F45" t="n">
+        <v>24</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.2544</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.1674</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0.7307</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0.2792</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0.207</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0.8571</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SC2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>BenLuc+CauNoi+TanAn</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>BenLuc</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>24</v>
+      </c>
+      <c r="F46" t="n">
+        <v>48</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.3027</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.1946</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0.6162</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0.4356</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0.2913</v>
+      </c>
+      <c r="L46" t="n">
+        <v>0.6504</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SC2</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>BenLuc+CauNoi+TanAn</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>BenLuc</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>48</v>
+      </c>
+      <c r="F47" t="n">
+        <v>12</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.2687</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.1827</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0.6976</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0.2777</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0.2027</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0.8583</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SC2</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>BenLuc+CauNoi+TanAn</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>BenLuc</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>48</v>
+      </c>
+      <c r="F48" t="n">
+        <v>24</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.2496</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.1653</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0.738</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0.2814</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0.2082</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0.8541</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SC2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>BenLuc+CauNoi+TanAn</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>BenLuc</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>48</v>
+      </c>
+      <c r="F49" t="n">
+        <v>48</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.3165</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.2091</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0.5759</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0.424</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0.2875</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0.6667999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>